<commit_message>
/HARDWARE/PRODUCTION: added production files for the next respin
</commit_message>
<xml_diff>
--- a/Hardware/production/bom.xlsx
+++ b/Hardware/production/bom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saleh\Desktop\Saleh Uni\sem 7\senior year project\Flight Controller\Hardware\production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33847371-59B8-4B87-86ED-48D86021C1CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A1F6F8B-F559-4BA8-B6B2-4B26FAC07151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="720" windowWidth="19200" windowHeight="11170" xr2:uid="{36651338-4E53-449A-911D-AA34483D6FC3}"/>
+    <workbookView xWindow="1060" yWindow="1060" windowWidth="19200" windowHeight="11170" xr2:uid="{2138F2A2-E1ED-4C96-B265-79A572D2D8F0}"/>
   </bookViews>
   <sheets>
     <sheet name="bom" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="175">
   <si>
     <t>Designator</t>
   </si>
@@ -40,9 +40,6 @@
     <t>C1, C10, C3</t>
   </si>
   <si>
-    <t>0603</t>
-  </si>
-  <si>
     <t>10uF</t>
   </si>
   <si>
@@ -73,9 +70,6 @@
     <t>C2, C24, C25, C26, C28, C29, C31, C32, C36, C37, C43, C44, C46, C5, C50, C51, C52, C53, C54, C55</t>
   </si>
   <si>
-    <t>0402</t>
-  </si>
-  <si>
     <t>C21</t>
   </si>
   <si>
@@ -100,9 +94,6 @@
     <t>C4</t>
   </si>
   <si>
-    <t>0805</t>
-  </si>
-  <si>
     <t>C45, C47</t>
   </si>
   <si>
@@ -304,9 +295,6 @@
     <t>R25, R26</t>
   </si>
   <si>
-    <t>R28</t>
-  </si>
-  <si>
     <t>R29, R30</t>
   </si>
   <si>
@@ -359,6 +347,81 @@
   </si>
   <si>
     <t>MCU_BOOT</t>
+  </si>
+  <si>
+    <t>TP1, TP10, TP12, TP17, TP18, TP21, TP22, TP25, TP26, TP27, TP4, TP43, TP45, TP6</t>
+  </si>
+  <si>
+    <t>Solderpad</t>
+  </si>
+  <si>
+    <t>power</t>
+  </si>
+  <si>
+    <t>TP13, TP16, TP20, TP24</t>
+  </si>
+  <si>
+    <t>servos</t>
+  </si>
+  <si>
+    <t>TP14, TP23</t>
+  </si>
+  <si>
+    <t>BAT pad</t>
+  </si>
+  <si>
+    <t>TP15</t>
+  </si>
+  <si>
+    <t>M4</t>
+  </si>
+  <si>
+    <t>TP2</t>
+  </si>
+  <si>
+    <t>Motor 1</t>
+  </si>
+  <si>
+    <t>TP28, TP33, TP34, TP35, TP36, TP37, TP38, TP39, TP40, TP41, TP42</t>
+  </si>
+  <si>
+    <t>sensors</t>
+  </si>
+  <si>
+    <t>TP29</t>
+  </si>
+  <si>
+    <t>TELEMETRY_RX</t>
+  </si>
+  <si>
+    <t>TP3, TP32, TP7, TP9</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>TP30</t>
+  </si>
+  <si>
+    <t>TELEMETRY_TX</t>
+  </si>
+  <si>
+    <t>TP31</t>
+  </si>
+  <si>
+    <t>5V</t>
+  </si>
+  <si>
+    <t>TP5</t>
+  </si>
+  <si>
+    <t>Motor 2</t>
+  </si>
+  <si>
+    <t>TP8</t>
+  </si>
+  <si>
+    <t>M3</t>
   </si>
   <si>
     <t>U1</t>
@@ -965,9 +1028,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1342,15 +1404,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65CCA22E-4277-4CFB-8799-771EC916E685}">
-  <dimension ref="A1:E77"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19797046-AE4D-4F0B-9C24-01AE2412D100}">
+  <dimension ref="A1:E76"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="83.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="47.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1373,504 +1429,504 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
+      <c r="B2">
+        <v>603</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>603</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>603</v>
       </c>
       <c r="C4">
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>603</v>
       </c>
       <c r="C5">
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>603</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
         <v>14</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>402</v>
       </c>
       <c r="C7">
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>603</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>6</v>
+        <v>18</v>
+      </c>
+      <c r="B9">
+        <v>603</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
+      </c>
+      <c r="B10">
+        <v>402</v>
       </c>
       <c r="C10">
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
+      </c>
+      <c r="B11">
+        <v>603</v>
       </c>
       <c r="C11">
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
+      </c>
+      <c r="B12">
+        <v>805</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>17</v>
+        <v>24</v>
+      </c>
+      <c r="B13">
+        <v>402</v>
       </c>
       <c r="C13">
         <v>2</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>17</v>
+        <v>26</v>
+      </c>
+      <c r="B14">
+        <v>402</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>17</v>
+        <v>28</v>
+      </c>
+      <c r="B15">
+        <v>402</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" t="s">
         <v>35</v>
-      </c>
-      <c r="B17" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>26</v>
+        <v>39</v>
+      </c>
+      <c r="B19">
+        <v>805</v>
       </c>
       <c r="C19">
         <v>4</v>
       </c>
       <c r="D19" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>47</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
+      </c>
+      <c r="B21">
+        <v>603</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C22">
         <v>4</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C24">
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B25" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
         <v>56</v>
-      </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-      <c r="D25" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B30" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C30">
         <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B31" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C32">
         <v>1</v>
       </c>
       <c r="D32" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B33" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B34" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C34">
         <v>1</v>
       </c>
       <c r="D34" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B35" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C35">
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E35" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>85</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>17</v>
+        <v>82</v>
+      </c>
+      <c r="B36">
+        <v>402</v>
       </c>
       <c r="C36">
         <v>2</v>
       </c>
       <c r="D36" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>87</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>17</v>
+        <v>84</v>
+      </c>
+      <c r="B37">
+        <v>402</v>
       </c>
       <c r="C37">
         <v>4</v>
@@ -1881,24 +1937,24 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>88</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>17</v>
+        <v>85</v>
+      </c>
+      <c r="B38">
+        <v>402</v>
       </c>
       <c r="C38">
         <v>5</v>
       </c>
       <c r="D38" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>90</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>17</v>
+        <v>87</v>
+      </c>
+      <c r="B39">
+        <v>402</v>
       </c>
       <c r="C39">
         <v>3</v>
@@ -1909,24 +1965,24 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>91</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>17</v>
+        <v>88</v>
+      </c>
+      <c r="B40">
+        <v>402</v>
       </c>
       <c r="C40">
         <v>4</v>
       </c>
       <c r="D40" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>93</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>17</v>
+        <v>90</v>
+      </c>
+      <c r="B41">
+        <v>402</v>
       </c>
       <c r="C41">
         <v>2</v>
@@ -1937,344 +1993,498 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>94</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>17</v>
+        <v>91</v>
+      </c>
+      <c r="B42">
+        <v>402</v>
       </c>
       <c r="C42">
-        <v>1</v>
-      </c>
-      <c r="D42">
-        <v>120</v>
+        <v>2</v>
+      </c>
+      <c r="D42" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>95</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>17</v>
+        <v>93</v>
+      </c>
+      <c r="B43">
+        <v>402</v>
       </c>
       <c r="C43">
         <v>2</v>
       </c>
       <c r="D43" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>97</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>17</v>
+        <v>95</v>
+      </c>
+      <c r="B44">
+        <v>402</v>
       </c>
       <c r="C44">
-        <v>2</v>
-      </c>
-      <c r="D44" t="s">
-        <v>98</v>
+        <v>1</v>
+      </c>
+      <c r="D44">
+        <v>49.9</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>99</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>17</v>
+        <v>96</v>
+      </c>
+      <c r="B45">
+        <v>402</v>
       </c>
       <c r="C45">
         <v>1</v>
       </c>
-      <c r="D45">
-        <v>49.9</v>
+      <c r="D45" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>100</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>17</v>
+        <v>98</v>
+      </c>
+      <c r="B46">
+        <v>402</v>
       </c>
       <c r="C46">
         <v>1</v>
       </c>
       <c r="D46" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>102</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>17</v>
+        <v>100</v>
+      </c>
+      <c r="B47">
+        <v>402</v>
       </c>
       <c r="C47">
         <v>1</v>
       </c>
       <c r="D47" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>104</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>17</v>
+        <v>102</v>
+      </c>
+      <c r="B48">
+        <v>402</v>
       </c>
       <c r="C48">
         <v>1</v>
       </c>
       <c r="D48" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
+        <v>104</v>
+      </c>
+      <c r="B49" t="s">
+        <v>105</v>
+      </c>
+      <c r="C49">
+        <v>1</v>
+      </c>
+      <c r="D49" t="s">
         <v>106</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C49">
-        <v>1</v>
-      </c>
-      <c r="D49" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
+        <v>107</v>
+      </c>
+      <c r="B50" t="s">
+        <v>105</v>
+      </c>
+      <c r="C50">
+        <v>1</v>
+      </c>
+      <c r="D50" t="s">
         <v>108</v>
-      </c>
-      <c r="B50" t="s">
-        <v>109</v>
-      </c>
-      <c r="C50">
-        <v>1</v>
-      </c>
-      <c r="D50" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>109</v>
+      </c>
+      <c r="B51" t="s">
+        <v>110</v>
+      </c>
+      <c r="C51">
+        <v>14</v>
+      </c>
+      <c r="D51" t="s">
         <v>111</v>
       </c>
-      <c r="B51" t="s">
-        <v>109</v>
-      </c>
-      <c r="C51">
-        <v>1</v>
-      </c>
-      <c r="D51" t="s">
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>112</v>
+      </c>
+      <c r="B52" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52">
+        <v>4</v>
+      </c>
+      <c r="D52" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>114</v>
+      </c>
+      <c r="B53" t="s">
+        <v>115</v>
+      </c>
+      <c r="C53">
+        <v>2</v>
+      </c>
+      <c r="D53" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>116</v>
+      </c>
+      <c r="B54" t="s">
+        <v>110</v>
+      </c>
+      <c r="C54">
+        <v>1</v>
+      </c>
+      <c r="D54" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>118</v>
+      </c>
+      <c r="B55" t="s">
+        <v>110</v>
+      </c>
+      <c r="C55">
+        <v>1</v>
+      </c>
+      <c r="D55" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>120</v>
+      </c>
+      <c r="B56" t="s">
+        <v>110</v>
+      </c>
+      <c r="C56">
+        <v>11</v>
+      </c>
+      <c r="D56" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>122</v>
+      </c>
+      <c r="B57" t="s">
+        <v>110</v>
+      </c>
+      <c r="C57">
+        <v>1</v>
+      </c>
+      <c r="D57" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>124</v>
+      </c>
+      <c r="B58" t="s">
+        <v>110</v>
+      </c>
+      <c r="C58">
+        <v>4</v>
+      </c>
+      <c r="D58" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>126</v>
+      </c>
+      <c r="B59" t="s">
+        <v>110</v>
+      </c>
+      <c r="C59">
+        <v>1</v>
+      </c>
+      <c r="D59" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>128</v>
+      </c>
+      <c r="B60" t="s">
+        <v>110</v>
+      </c>
+      <c r="C60">
+        <v>1</v>
+      </c>
+      <c r="D60" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>130</v>
+      </c>
+      <c r="B61" t="s">
+        <v>110</v>
+      </c>
+      <c r="C61">
+        <v>1</v>
+      </c>
+      <c r="D61" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>132</v>
+      </c>
+      <c r="B62" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62">
+        <v>1</v>
+      </c>
+      <c r="D62" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>134</v>
+      </c>
+      <c r="B63" t="s">
+        <v>135</v>
+      </c>
+      <c r="C63">
+        <v>1</v>
+      </c>
+      <c r="D63" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="B64" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="C64">
         <v>1</v>
       </c>
       <c r="D64" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="B65" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C65">
         <v>1</v>
       </c>
       <c r="D65" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="B66" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="C66">
         <v>1</v>
       </c>
       <c r="D66" t="s">
-        <v>121</v>
+        <v>144</v>
+      </c>
+      <c r="E66" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>122</v>
+        <v>146</v>
       </c>
       <c r="B67" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="C67">
         <v>1</v>
       </c>
       <c r="D67" t="s">
-        <v>123</v>
-      </c>
-      <c r="E67" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="B68" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="C68">
         <v>1</v>
       </c>
       <c r="D68" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B69" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="C69">
         <v>1</v>
       </c>
       <c r="D69" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="B70" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="C70">
         <v>1</v>
       </c>
       <c r="D70" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="B71" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="C71">
         <v>1</v>
       </c>
       <c r="D71" t="s">
-        <v>135</v>
+        <v>159</v>
+      </c>
+      <c r="E71" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="B72" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="C72">
         <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>138</v>
-      </c>
-      <c r="E72" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="B73" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="C73">
         <v>1</v>
       </c>
       <c r="D73" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="B74" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="C74">
         <v>1</v>
       </c>
       <c r="D74" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="B75" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="C75">
         <v>1</v>
       </c>
       <c r="D75" t="s">
-        <v>147</v>
+        <v>171</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="B76" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
       <c r="C76">
         <v>1</v>
       </c>
       <c r="D76" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>151</v>
-      </c>
-      <c r="B77" t="s">
-        <v>152</v>
-      </c>
-      <c r="C77">
-        <v>1</v>
-      </c>
-      <c r="D77" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>